<commit_message>
Ay sonu haftası eklendi, keyword-grafik atlaması ve mobil içindekiler düzeltildi
- Geçmiş aylarda Trends penceresi ayın son gününü içeren haftada bitiyor
  (Mar, Nis, May, Haz, Tem, Ağu yeniden çekildi; Temmuz 26 Tem - 1 Ağu)
- Keyword'e tıklayınca sayfa kart kabına kayıyor; filtre açıkken hedef
  kart görünür oluyor; keskin yükselişler tablosu da karta bağlı
- 1080 px altında içindekiler: yüzen düğme + alttan açılan panel
- bere, Mayıs 2025 tek seferlik sıçramasından dolayı 'bere modelleri'
  vekiliyle ölçülüyor

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aralik/ozdilekteyim-aralik-2026-arama-talebi.xlsx
+++ b/aralik/ozdilekteyim-aralik-2026-arama-talebi.xlsx
@@ -3893,17 +3893,23 @@
         <v>0</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="J63" s="10" t="n">
-        <v>0.09090909090909091</v>
-      </c>
-      <c r="K63" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="J63" s="5" t="n">
         <v>-0.2</v>
       </c>
-      <c r="L63" s="4" t="inlineStr"/>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L63" s="4" t="inlineStr">
+        <is>
+          <t>bere modelleri</t>
+        </is>
+      </c>
       <c r="M63" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N63" s="4" t="inlineStr">
         <is>
@@ -22797,141 +22803,145 @@
           <t>bere</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr"/>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>bere modelleri</t>
+        </is>
+      </c>
       <c r="C63" s="3" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H63" s="3" t="n">
         <v>24</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L63" s="3" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>31</v>
       </c>
       <c r="N63" s="3" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="O63" s="3" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="P63" s="3" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>100</v>
       </c>
       <c r="S63" s="3" t="n">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="T63" s="3" t="n">
-        <v>64</v>
+        <v>86</v>
       </c>
       <c r="U63" s="3" t="n">
-        <v>67</v>
+        <v>96</v>
       </c>
       <c r="V63" s="3" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="W63" s="3" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="X63" s="3" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="Y63" s="3" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="Z63" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="AA63" s="3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AB63" s="3" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="AC63" s="3" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="AD63" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="AE63" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="AE63" s="3" t="n">
-        <v>12</v>
-      </c>
       <c r="AF63" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AG63" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AH63" s="3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="AI63" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AJ63" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AK63" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AL63" s="3" t="n">
         <v>9</v>
       </c>
       <c r="AM63" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="AN63" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AO63" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="AP63" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="AN63" s="3" t="n">
+      <c r="AQ63" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="AR63" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="AO63" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="AP63" s="3" t="n">
+      <c r="AS63" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="AQ63" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="AR63" s="3" t="n">
+      <c r="AT63" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AU63" s="3" t="n">
         <v>10</v>
-      </c>
-      <c r="AS63" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="AT63" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="AU63" s="3" t="n">
-        <v>12</v>
       </c>
       <c r="AV63" s="3" t="n">
         <v>11</v>
@@ -22943,19 +22953,19 @@
         <v>10</v>
       </c>
       <c r="AY63" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AZ63" s="3" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="BA63" s="3" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="BB63" s="3" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="BC63" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="64">

</xml_diff>